<commit_message>
Add/Update Positions2.xlsx via API
</commit_message>
<xml_diff>
--- a/ETF/Positions2.xlsx
+++ b/ETF/Positions2.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1001"/>
+  <dimension ref="A1:D1003"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14456,6 +14456,34 @@
         <v>161883.6181671875</v>
       </c>
     </row>
+    <row r="1002">
+      <c r="A1002" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B1002" t="n">
+        <v>157912.1221998047</v>
+      </c>
+      <c r="C1002" t="n">
+        <v>2744.15</v>
+      </c>
+      <c r="D1002" t="n">
+        <v>160656.2721998047</v>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B1003" t="n">
+        <v>157912.1221998047</v>
+      </c>
+      <c r="C1003" t="n">
+        <v>2744.15</v>
+      </c>
+      <c r="D1003" t="n">
+        <v>160656.2721998047</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>